<commit_message>
Dealer import by product code with FIFO allocation + sale date
</commit_message>
<xml_diff>
--- a/public/mau-import-ban-dai-ly.xlsx
+++ b/public/mau-import-ban-dai-ly.xlsx
@@ -406,7 +406,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>MaLo</v>
+        <v>MaHang</v>
       </c>
       <c r="B1" t="str">
         <v>SoLuong</v>
@@ -417,7 +417,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>OWN-2610-0001</v>
+        <v>AZ1664430120-SMS-30759</v>
       </c>
       <c r="B2">
         <v>10</v>
@@ -428,7 +428,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>OWN-2610-0002</v>
+        <v>AZ1664440069-SMS-30705</v>
       </c>
       <c r="B3">
         <v>5</v>

</xml_diff>

<commit_message>
Import ban hang theo ten + dong xe: STT, Dong xe, Ten phu tung, So luong, Don gia; gia mac dinh theo loai khach (le/gara/dai ly); MaHang tuy chon khi trung ten; FIFO + ngay ban khong doi
</commit_message>
<xml_diff>
--- a/public/mau-import-ban-dai-ly.xlsx
+++ b/public/mau-import-ban-dai-ly.xlsx
@@ -397,49 +397,69 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:E3"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
     <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="20.83203125" customWidth="1"/>
+    <col min="5" max="5" width="20.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>MaHang</v>
+        <v>STT</v>
       </c>
       <c r="B1" t="str">
-        <v>SoLuong</v>
+        <v>Dòng xe</v>
       </c>
       <c r="C1" t="str">
-        <v>DonGiaVND</v>
+        <v>Tên phụ tùng</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Số lượng</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Đơn giá</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
-        <v>AZ1664430120-SMS-30759</v>
-      </c>
-      <c r="B2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>420</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Bầu hơi cabin trước</v>
+      </c>
+      <c r="D2">
         <v>10</v>
       </c>
-      <c r="C2" t="str">
+      <c r="E2" t="str">
         <v/>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
-        <v>AZ1664440069-SMS-30705</v>
-      </c>
-      <c r="B3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>420</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Bầu hơi cabin sau</v>
+      </c>
+      <c r="D3">
         <v>5</v>
       </c>
-      <c r="C3">
+      <c r="E3">
         <v>1200000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ban hang theo ma san pham: import ban hang bat buoc MaHang, trung ten khac ma van ban dung; chuan hoa ma bo khoang trang
</commit_message>
<xml_diff>
--- a/public/mau-import-ban-dai-ly.xlsx
+++ b/public/mau-import-ban-dai-ly.xlsx
@@ -397,13 +397,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:F5"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
     <col min="3" max="3" width="20.83203125" customWidth="1"/>
     <col min="4" max="4" width="20.83203125" customWidth="1"/>
     <col min="5" max="5" width="20.83203125" customWidth="1"/>
+    <col min="6" max="6" width="20.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -411,15 +412,18 @@
         <v>STT</v>
       </c>
       <c r="B1" t="str">
+        <v>Mã hàng</v>
+      </c>
+      <c r="C1" t="str">
         <v>Dòng xe</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>Tên phụ tùng</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>Số lượng</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Đơn giá</v>
       </c>
     </row>
@@ -428,15 +432,18 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
+        <v>AZ1664430120-SMS-30759</v>
+      </c>
+      <c r="C2" t="str">
         <v>420</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v>Bầu hơi cabin trước</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>10</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v/>
       </c>
     </row>
@@ -445,21 +452,64 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
+        <v>AZ1664440069-SMS-30705</v>
+      </c>
+      <c r="C3" t="str">
         <v>420</v>
       </c>
-      <c r="C3" t="str">
+      <c r="D3" t="str">
         <v>Bầu hơi cabin sau</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>5</v>
       </c>
-      <c r="E3">
+      <c r="F3">
+        <v>1200000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>VG1540080110-CX1020 SMS-10452</v>
+      </c>
+      <c r="C4" t="str">
+        <v>420</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Lọc dầu</v>
+      </c>
+      <c r="E4">
+        <v>10</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>WG1540080211-CX1017 SMS10453</v>
+      </c>
+      <c r="C5" t="str">
+        <v>420</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Lọc dầu</v>
+      </c>
+      <c r="E5">
+        <v>5</v>
+      </c>
+      <c r="F5">
         <v>1200000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>